<commit_message>
feat: add Moya Semya command support with family stats parsing and monitoring
</commit_message>
<xml_diff>
--- a/Команды распознание.xlsx
+++ b/Команды распознание.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Toxa\Desktop\VK\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F81F14-510A-4A6F-971B-459A7C24A480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39D8AE66-6402-43E0-8F6F-EA2A8AAE98A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="104">
   <si>
     <t>Команды Жабабота</t>
   </si>
@@ -340,6 +340,12 @@
   </si>
   <si>
     <t>+</t>
+  </si>
+  <si>
+    <t>В процессе</t>
+  </si>
+  <si>
+    <t>Доделать распознавание. Надо делать уже после огорода, чтобы добавить выпадающие семена</t>
   </si>
 </sst>
 </file>
@@ -827,7 +833,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -835,7 +841,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C7" t="s">
         <v>101</v>
@@ -857,7 +863,7 @@
         <v>67</v>
       </c>
       <c r="B9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -984,7 +990,7 @@
         <v>17</v>
       </c>
       <c r="B26" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
feat: add parser_type classification, response_type handling, delta audit tab, description column
- Classify commands into 3 parser types: control, simple, additive
- Connect response_type (success/cooldown/error) in regex-parsing branch
- Add parser_type color badge in recognition accordion UI
- Add 'Аудит дельт' tab with API endpoints (recognition.db)
- Add description column to monitored_commands with seed data
- Add inline description editing in UI
- Update all documentation (.md files)
</commit_message>
<xml_diff>
--- a/Команды распознание.xlsx
+++ b/Команды распознание.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Toxa\Desktop\VK\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39D8AE66-6402-43E0-8F6F-EA2A8AAE98A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DE7E09F-9411-42F8-B260-F2771D4BB96F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Команды Жабабота" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Команды Жабабота'!$A$1:$B$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Команды Жабабота'!$A$1:$B$98</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="105">
   <si>
     <t>Команды Жабабота</t>
   </si>
@@ -342,10 +342,13 @@
     <t>+</t>
   </si>
   <si>
-    <t>В процессе</t>
-  </si>
-  <si>
     <t>Доделать распознавание. Надо делать уже после огорода, чтобы добавить выпадающие семена</t>
+  </si>
+  <si>
+    <t>Открыть стоп-лист</t>
+  </si>
+  <si>
+    <t>ваываы</t>
   </si>
 </sst>
 </file>
@@ -781,7 +784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="80" customWidth="1"/>
@@ -833,7 +836,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -841,7 +844,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C7" t="s">
         <v>101</v>
@@ -990,7 +993,7 @@
         <v>17</v>
       </c>
       <c r="B26" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -1271,7 +1274,7 @@
         <v>33</v>
       </c>
       <c r="B63" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -1546,8 +1549,17 @@
         <v>99</v>
       </c>
     </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A98" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B98" t="s">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B97" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:B98" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>